<commit_message>
Fill blank start and deadline dates from the source file.
Keep a date already shown in the client sample, and take the source date only when that cell was empty.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Ready_UT_PO_STATUS_13.10.2026.xlsx
+++ b/Ready_UT_PO_STATUS_13.10.2026.xlsx
@@ -893,11 +893,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K3" s="15" t="n"/>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>07.10.2026</t>
+        </is>
+      </c>
       <c r="L3" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="M3" s="8" t="n"/>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>16.11.2026</t>
+        </is>
+      </c>
       <c r="N3" s="15" t="n"/>
       <c r="O3" s="15" t="inlineStr">
         <is>
@@ -962,11 +970,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K4" s="15" t="n"/>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>12.10.2026</t>
+        </is>
+      </c>
       <c r="L4" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M4" s="8" t="n"/>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>11.11.2026</t>
+        </is>
+      </c>
       <c r="N4" s="15" t="n"/>
       <c r="O4" s="15" t="inlineStr">
         <is>
@@ -1031,11 +1047,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K5" s="15" t="n"/>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>13.10.2026</t>
+        </is>
+      </c>
       <c r="L5" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="M5" s="8" t="n"/>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>22.11.2026</t>
+        </is>
+      </c>
       <c r="N5" s="15" t="n"/>
       <c r="O5" s="15" t="inlineStr">
         <is>
@@ -1100,11 +1124,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K6" s="15" t="n"/>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>13.10.2026</t>
+        </is>
+      </c>
       <c r="L6" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M6" s="8" t="n"/>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>12.11.2026</t>
+        </is>
+      </c>
       <c r="N6" s="15" t="n"/>
       <c r="O6" s="15" t="inlineStr">
         <is>
@@ -1169,11 +1201,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K7" s="15" t="n"/>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>13.10.2026</t>
+        </is>
+      </c>
       <c r="L7" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M7" s="8" t="n"/>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>12.11.2026</t>
+        </is>
+      </c>
       <c r="N7" s="15" t="n"/>
       <c r="O7" s="15" t="inlineStr">
         <is>
@@ -1272,11 +1312,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K9" s="15" t="n"/>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L9" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M9" s="8" t="n"/>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>29.10.2026</t>
+        </is>
+      </c>
       <c r="N9" s="15" t="n"/>
       <c r="O9" s="15" t="inlineStr">
         <is>
@@ -1349,11 +1397,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K10" s="15" t="n"/>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>12.08.2026</t>
+        </is>
+      </c>
       <c r="L10" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="M10" s="8" t="n"/>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>06.09.2026</t>
+        </is>
+      </c>
       <c r="N10" s="15" t="n"/>
       <c r="O10" s="15" t="inlineStr">
         <is>
@@ -2270,11 +2326,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K22" s="15" t="n"/>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>22.07.2026</t>
+        </is>
+      </c>
       <c r="L22" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="M22" s="8" t="n"/>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>16.08.2026</t>
+        </is>
+      </c>
       <c r="N22" s="15" t="n"/>
       <c r="O22" s="15" t="inlineStr">
         <is>
@@ -2344,11 +2408,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K23" s="15" t="n"/>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
       <c r="L23" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="M23" s="8" t="n"/>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t>10.09.2026</t>
+        </is>
+      </c>
       <c r="N23" s="15" t="n"/>
       <c r="O23" s="15" t="inlineStr">
         <is>
@@ -4842,11 +4914,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K55" s="15" t="n"/>
+      <c r="K55" s="15" t="inlineStr">
+        <is>
+          <t>01.10.2026</t>
+        </is>
+      </c>
       <c r="L55" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M55" s="8" t="n"/>
+      <c r="M55" s="8" t="inlineStr">
+        <is>
+          <t>31.10.2026</t>
+        </is>
+      </c>
       <c r="N55" s="15" t="n"/>
       <c r="O55" s="15" t="inlineStr">
         <is>
@@ -4923,11 +5003,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K56" s="15" t="n"/>
+      <c r="K56" s="15" t="inlineStr">
+        <is>
+          <t>25.09.2026</t>
+        </is>
+      </c>
       <c r="L56" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="M56" s="8" t="n"/>
+      <c r="M56" s="8" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
       <c r="N56" s="15" t="n"/>
       <c r="O56" s="15" t="inlineStr">
         <is>
@@ -5000,11 +5088,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K57" s="15" t="n"/>
+      <c r="K57" s="15" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L57" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M57" s="8" t="n"/>
+      <c r="M57" s="8" t="inlineStr">
+        <is>
+          <t>29.10.2026</t>
+        </is>
+      </c>
       <c r="N57" s="15" t="n"/>
       <c r="O57" s="15" t="inlineStr">
         <is>
@@ -5077,11 +5173,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K58" s="15" t="n"/>
+      <c r="K58" s="15" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L58" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M58" s="8" t="n"/>
+      <c r="M58" s="8" t="inlineStr">
+        <is>
+          <t>29.10.2026</t>
+        </is>
+      </c>
       <c r="N58" s="15" t="n"/>
       <c r="O58" s="15" t="inlineStr">
         <is>
@@ -5154,11 +5258,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K59" s="15" t="n"/>
+      <c r="K59" s="15" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
       <c r="L59" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M59" s="8" t="n"/>
+      <c r="M59" s="8" t="inlineStr">
+        <is>
+          <t>29.10.2026</t>
+        </is>
+      </c>
       <c r="N59" s="15" t="n"/>
       <c r="O59" s="15" t="inlineStr">
         <is>
@@ -5231,11 +5343,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K60" s="15" t="n"/>
+      <c r="K60" s="15" t="inlineStr">
+        <is>
+          <t>11.09.2026</t>
+        </is>
+      </c>
       <c r="L60" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="M60" s="8" t="n"/>
+      <c r="M60" s="8" t="inlineStr">
+        <is>
+          <t>23.10.2026</t>
+        </is>
+      </c>
       <c r="N60" s="15" t="n"/>
       <c r="O60" s="15" t="inlineStr">
         <is>
@@ -8665,7 +8785,11 @@
           <t>04.09.2026</t>
         </is>
       </c>
-      <c r="N100" s="15" t="n"/>
+      <c r="N100" s="15" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
       <c r="O100" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -8842,7 +8966,11 @@
           <t>04.09.2026</t>
         </is>
       </c>
-      <c r="N102" s="15" t="n"/>
+      <c r="N102" s="15" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
       <c r="O102" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -8928,7 +9056,11 @@
           <t>03.09.2026</t>
         </is>
       </c>
-      <c r="N103" s="15" t="n"/>
+      <c r="N103" s="15" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
       <c r="O103" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -9821,7 +9953,11 @@
           <t>19.07.2026</t>
         </is>
       </c>
-      <c r="N113" s="15" t="n"/>
+      <c r="N113" s="15" t="inlineStr">
+        <is>
+          <t>21.08.2026</t>
+        </is>
+      </c>
       <c r="O113" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -9903,7 +10039,11 @@
           <t>19.07.2026</t>
         </is>
       </c>
-      <c r="N114" s="15" t="n"/>
+      <c r="N114" s="15" t="inlineStr">
+        <is>
+          <t>21.08.2026</t>
+        </is>
+      </c>
       <c r="O114" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -38695,11 +38835,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K437" s="15" t="n"/>
+      <c r="K437" s="15" t="inlineStr">
+        <is>
+          <t>26.03.2026</t>
+        </is>
+      </c>
       <c r="L437" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M437" s="8" t="n"/>
+      <c r="M437" s="8" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
       <c r="N437" s="15" t="inlineStr">
         <is>
           <t>27.05.2026</t>
@@ -38974,11 +39122,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K441" s="15" t="n"/>
+      <c r="K441" s="15" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
       <c r="L441" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="M441" s="8" t="n"/>
+      <c r="M441" s="8" t="inlineStr">
+        <is>
+          <t>06.08.2026</t>
+        </is>
+      </c>
       <c r="N441" s="15" t="n"/>
       <c r="O441" s="15" t="inlineStr">
         <is>
@@ -39043,11 +39199,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K442" s="15" t="n"/>
+      <c r="K442" s="15" t="inlineStr">
+        <is>
+          <t>12.08.2026</t>
+        </is>
+      </c>
       <c r="L442" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="M442" s="8" t="n"/>
+      <c r="M442" s="8" t="inlineStr">
+        <is>
+          <t>06.09.2026</t>
+        </is>
+      </c>
       <c r="N442" s="15" t="n"/>
       <c r="O442" s="15" t="inlineStr">
         <is>
@@ -42788,11 +42952,19 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K486" s="15" t="n"/>
+      <c r="K486" s="15" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
       <c r="L486" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M486" s="8" t="n"/>
+      <c r="M486" s="8" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
       <c r="N486" s="15" t="n"/>
       <c r="O486" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Leave awaiting-advance rows without dates.
Start, deadline, planned, and actual dates stay empty in that section. Other sections still take a blank date from the source file.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Ready_UT_PO_STATUS_13.10.2026.xlsx
+++ b/Ready_UT_PO_STATUS_13.10.2026.xlsx
@@ -893,19 +893,11 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K3" s="15" t="inlineStr">
-        <is>
-          <t>07.10.2026</t>
-        </is>
-      </c>
+      <c r="K3" s="15" t="n"/>
       <c r="L3" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>16.11.2026</t>
-        </is>
-      </c>
+      <c r="M3" s="8" t="n"/>
       <c r="N3" s="15" t="n"/>
       <c r="O3" s="15" t="inlineStr">
         <is>
@@ -970,19 +962,11 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K4" s="15" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+      <c r="K4" s="15" t="n"/>
       <c r="L4" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M4" s="8" t="inlineStr">
-        <is>
-          <t>11.11.2026</t>
-        </is>
-      </c>
+      <c r="M4" s="8" t="n"/>
       <c r="N4" s="15" t="n"/>
       <c r="O4" s="15" t="inlineStr">
         <is>
@@ -1047,19 +1031,11 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K5" s="15" t="inlineStr">
-        <is>
-          <t>13.10.2026</t>
-        </is>
-      </c>
+      <c r="K5" s="15" t="n"/>
       <c r="L5" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>22.11.2026</t>
-        </is>
-      </c>
+      <c r="M5" s="8" t="n"/>
       <c r="N5" s="15" t="n"/>
       <c r="O5" s="15" t="inlineStr">
         <is>
@@ -1124,19 +1100,11 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K6" s="15" t="inlineStr">
-        <is>
-          <t>13.10.2026</t>
-        </is>
-      </c>
+      <c r="K6" s="15" t="n"/>
       <c r="L6" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M6" s="8" t="inlineStr">
-        <is>
-          <t>12.11.2026</t>
-        </is>
-      </c>
+      <c r="M6" s="8" t="n"/>
       <c r="N6" s="15" t="n"/>
       <c r="O6" s="15" t="inlineStr">
         <is>
@@ -1201,19 +1169,11 @@
           <t>EA</t>
         </is>
       </c>
-      <c r="K7" s="15" t="inlineStr">
-        <is>
-          <t>13.10.2026</t>
-        </is>
-      </c>
+      <c r="K7" s="15" t="n"/>
       <c r="L7" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="M7" s="8" t="inlineStr">
-        <is>
-          <t>12.11.2026</t>
-        </is>
-      </c>
+      <c r="M7" s="8" t="n"/>
       <c r="N7" s="15" t="n"/>
       <c r="O7" s="15" t="inlineStr">
         <is>

</xml_diff>